<commit_message>
Atualização automática diária da base
</commit_message>
<xml_diff>
--- a/base_despesas/2025/despesas_202512.xlsx
+++ b/base_despesas/2025/despesas_202512.xlsx
@@ -702,7 +702,7 @@
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -825,7 +825,7 @@
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -948,7 +948,7 @@
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1440,7 @@
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -1563,7 +1563,7 @@
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1686,7 @@
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -1809,7 +1809,7 @@
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -2178,7 +2178,7 @@
       </c>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="AG15" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2424,7 @@
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -2547,7 +2547,7 @@
       </c>
       <c r="AG17" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -2670,7 +2670,7 @@
       </c>
       <c r="AG18" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -2793,7 +2793,7 @@
       </c>
       <c r="AG19" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -2916,7 +2916,7 @@
       </c>
       <c r="AG20" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -3039,7 +3039,7 @@
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
       </c>
       <c r="AG22" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -3285,7 +3285,7 @@
       </c>
       <c r="AG23" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="AG24" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AG25" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -3654,7 +3654,7 @@
       </c>
       <c r="AG26" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -3777,7 +3777,7 @@
       </c>
       <c r="AG27" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="AG28" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="AG29" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="AG30" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -4269,7 +4269,7 @@
       </c>
       <c r="AG31" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -4392,7 +4392,7 @@
       </c>
       <c r="AG32" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -4515,7 +4515,7 @@
       </c>
       <c r="AG33" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -4638,7 +4638,7 @@
       </c>
       <c r="AG34" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -4761,7 +4761,7 @@
       </c>
       <c r="AG35" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -4884,7 +4884,7 @@
       </c>
       <c r="AG36" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -5007,7 +5007,7 @@
       </c>
       <c r="AG37" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AG38" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -5253,7 +5253,7 @@
       </c>
       <c r="AG39" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5376,7 @@
       </c>
       <c r="AG40" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -5499,7 +5499,7 @@
       </c>
       <c r="AG41" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -5622,7 +5622,7 @@
       </c>
       <c r="AG42" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -5745,7 +5745,7 @@
       </c>
       <c r="AG43" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -5868,7 +5868,7 @@
       </c>
       <c r="AG44" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -5991,7 +5991,7 @@
       </c>
       <c r="AG45" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -6114,7 +6114,7 @@
       </c>
       <c r="AG46" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -6237,7 +6237,7 @@
       </c>
       <c r="AG47" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -6360,7 +6360,7 @@
       </c>
       <c r="AG48" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -6483,7 +6483,7 @@
       </c>
       <c r="AG49" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -6606,7 +6606,7 @@
       </c>
       <c r="AG50" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="AG51" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -6852,7 +6852,7 @@
       </c>
       <c r="AG52" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -6975,7 +6975,7 @@
       </c>
       <c r="AG53" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -7098,7 +7098,7 @@
       </c>
       <c r="AG54" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -7221,7 +7221,7 @@
       </c>
       <c r="AG55" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -7344,7 +7344,7 @@
       </c>
       <c r="AG56" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -7467,7 +7467,7 @@
       </c>
       <c r="AG57" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -7590,7 +7590,7 @@
       </c>
       <c r="AG58" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -7713,7 +7713,7 @@
       </c>
       <c r="AG59" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -7836,7 +7836,7 @@
       </c>
       <c r="AG60" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -7959,7 +7959,7 @@
       </c>
       <c r="AG61" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -8082,7 +8082,7 @@
       </c>
       <c r="AG62" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -8205,7 +8205,7 @@
       </c>
       <c r="AG63" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -8328,7 +8328,7 @@
       </c>
       <c r="AG64" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -8451,7 +8451,7 @@
       </c>
       <c r="AG65" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -8574,7 +8574,7 @@
       </c>
       <c r="AG66" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -8697,7 +8697,7 @@
       </c>
       <c r="AG67" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -8820,7 +8820,7 @@
       </c>
       <c r="AG68" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -8943,7 +8943,7 @@
       </c>
       <c r="AG69" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -9066,7 +9066,7 @@
       </c>
       <c r="AG70" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -9189,7 +9189,7 @@
       </c>
       <c r="AG71" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -9312,7 +9312,7 @@
       </c>
       <c r="AG72" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -9435,7 +9435,7 @@
       </c>
       <c r="AG73" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -9558,7 +9558,7 @@
       </c>
       <c r="AG74" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -9681,7 +9681,7 @@
       </c>
       <c r="AG75" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -9804,7 +9804,7 @@
       </c>
       <c r="AG76" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -9927,7 +9927,7 @@
       </c>
       <c r="AG77" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -10050,7 +10050,7 @@
       </c>
       <c r="AG78" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -10173,7 +10173,7 @@
       </c>
       <c r="AG79" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -10296,7 +10296,7 @@
       </c>
       <c r="AG80" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -10419,7 +10419,7 @@
       </c>
       <c r="AG81" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -10542,7 +10542,7 @@
       </c>
       <c r="AG82" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -10665,7 +10665,7 @@
       </c>
       <c r="AG83" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -10788,7 +10788,7 @@
       </c>
       <c r="AG84" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -10911,7 +10911,7 @@
       </c>
       <c r="AG85" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -11034,7 +11034,7 @@
       </c>
       <c r="AG86" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -11157,7 +11157,7 @@
       </c>
       <c r="AG87" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -11280,7 +11280,7 @@
       </c>
       <c r="AG88" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -11403,7 +11403,7 @@
       </c>
       <c r="AG89" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -11526,7 +11526,7 @@
       </c>
       <c r="AG90" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -11649,7 +11649,7 @@
       </c>
       <c r="AG91" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -11772,7 +11772,7 @@
       </c>
       <c r="AG92" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -11895,7 +11895,7 @@
       </c>
       <c r="AG93" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -12018,7 +12018,7 @@
       </c>
       <c r="AG94" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -12141,7 +12141,7 @@
       </c>
       <c r="AG95" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -12264,7 +12264,7 @@
       </c>
       <c r="AG96" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -12387,7 +12387,7 @@
       </c>
       <c r="AG97" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -12510,7 +12510,7 @@
       </c>
       <c r="AG98" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -12633,7 +12633,7 @@
       </c>
       <c r="AG99" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -12756,7 +12756,7 @@
       </c>
       <c r="AG100" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -12879,7 +12879,7 @@
       </c>
       <c r="AG101" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -13002,7 +13002,7 @@
       </c>
       <c r="AG102" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -13125,7 +13125,7 @@
       </c>
       <c r="AG103" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -13248,7 +13248,7 @@
       </c>
       <c r="AG104" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -13371,7 +13371,7 @@
       </c>
       <c r="AG105" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -13494,7 +13494,7 @@
       </c>
       <c r="AG106" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -13617,7 +13617,7 @@
       </c>
       <c r="AG107" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -13740,7 +13740,7 @@
       </c>
       <c r="AG108" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -13863,7 +13863,7 @@
       </c>
       <c r="AG109" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -13986,7 +13986,7 @@
       </c>
       <c r="AG110" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -14109,7 +14109,7 @@
       </c>
       <c r="AG111" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -14232,7 +14232,7 @@
       </c>
       <c r="AG112" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -14355,7 +14355,7 @@
       </c>
       <c r="AG113" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -14478,7 +14478,7 @@
       </c>
       <c r="AG114" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -14601,7 +14601,7 @@
       </c>
       <c r="AG115" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -14724,7 +14724,7 @@
       </c>
       <c r="AG116" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -14847,7 +14847,7 @@
       </c>
       <c r="AG117" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -14970,7 +14970,7 @@
       </c>
       <c r="AG118" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -15093,7 +15093,7 @@
       </c>
       <c r="AG119" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -15216,7 +15216,7 @@
       </c>
       <c r="AG120" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -15339,7 +15339,7 @@
       </c>
       <c r="AG121" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -15462,7 +15462,7 @@
       </c>
       <c r="AG122" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -15585,7 +15585,7 @@
       </c>
       <c r="AG123" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -15708,7 +15708,7 @@
       </c>
       <c r="AG124" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -15831,7 +15831,7 @@
       </c>
       <c r="AG125" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -15954,7 +15954,7 @@
       </c>
       <c r="AG126" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -16077,7 +16077,7 @@
       </c>
       <c r="AG127" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -16200,7 +16200,7 @@
       </c>
       <c r="AG128" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -16323,7 +16323,7 @@
       </c>
       <c r="AG129" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -16446,7 +16446,7 @@
       </c>
       <c r="AG130" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -16569,7 +16569,7 @@
       </c>
       <c r="AG131" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -16692,7 +16692,7 @@
       </c>
       <c r="AG132" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -16815,7 +16815,7 @@
       </c>
       <c r="AG133" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -16938,7 +16938,7 @@
       </c>
       <c r="AG134" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -17061,7 +17061,7 @@
       </c>
       <c r="AG135" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -17184,7 +17184,7 @@
       </c>
       <c r="AG136" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -17307,7 +17307,7 @@
       </c>
       <c r="AG137" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -17430,7 +17430,7 @@
       </c>
       <c r="AG138" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -17553,7 +17553,7 @@
       </c>
       <c r="AG139" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -17676,7 +17676,7 @@
       </c>
       <c r="AG140" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -17799,7 +17799,7 @@
       </c>
       <c r="AG141" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -17922,7 +17922,7 @@
       </c>
       <c r="AG142" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -18045,7 +18045,7 @@
       </c>
       <c r="AG143" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -18168,7 +18168,7 @@
       </c>
       <c r="AG144" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -18291,7 +18291,7 @@
       </c>
       <c r="AG145" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -18414,7 +18414,7 @@
       </c>
       <c r="AG146" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -18537,7 +18537,7 @@
       </c>
       <c r="AG147" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -18660,7 +18660,7 @@
       </c>
       <c r="AG148" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -18783,7 +18783,7 @@
       </c>
       <c r="AG149" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -18906,7 +18906,7 @@
       </c>
       <c r="AG150" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -19029,7 +19029,7 @@
       </c>
       <c r="AG151" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -19152,7 +19152,7 @@
       </c>
       <c r="AG152" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -19275,7 +19275,7 @@
       </c>
       <c r="AG153" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -19398,7 +19398,7 @@
       </c>
       <c r="AG154" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -19521,7 +19521,7 @@
       </c>
       <c r="AG155" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -19644,7 +19644,7 @@
       </c>
       <c r="AG156" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -19767,7 +19767,7 @@
       </c>
       <c r="AG157" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -19890,7 +19890,7 @@
       </c>
       <c r="AG158" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -20013,7 +20013,7 @@
       </c>
       <c r="AG159" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -20136,7 +20136,7 @@
       </c>
       <c r="AG160" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -20259,7 +20259,7 @@
       </c>
       <c r="AG161" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -20382,7 +20382,7 @@
       </c>
       <c r="AG162" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -20505,7 +20505,7 @@
       </c>
       <c r="AG163" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -20628,7 +20628,7 @@
       </c>
       <c r="AG164" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -20751,7 +20751,7 @@
       </c>
       <c r="AG165" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -20874,7 +20874,7 @@
       </c>
       <c r="AG166" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -20997,7 +20997,7 @@
       </c>
       <c r="AG167" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -21120,7 +21120,7 @@
       </c>
       <c r="AG168" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -21243,7 +21243,7 @@
       </c>
       <c r="AG169" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -21366,7 +21366,7 @@
       </c>
       <c r="AG170" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -21489,7 +21489,7 @@
       </c>
       <c r="AG171" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -21612,7 +21612,7 @@
       </c>
       <c r="AG172" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -21735,7 +21735,7 @@
       </c>
       <c r="AG173" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -21858,7 +21858,7 @@
       </c>
       <c r="AG174" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -21981,7 +21981,7 @@
       </c>
       <c r="AG175" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -22104,7 +22104,7 @@
       </c>
       <c r="AG176" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -22227,7 +22227,7 @@
       </c>
       <c r="AG177" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -22350,7 +22350,7 @@
       </c>
       <c r="AG178" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -22473,7 +22473,7 @@
       </c>
       <c r="AG179" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -22596,7 +22596,7 @@
       </c>
       <c r="AG180" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -22719,7 +22719,7 @@
       </c>
       <c r="AG181" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -22842,7 +22842,7 @@
       </c>
       <c r="AG182" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -22965,7 +22965,7 @@
       </c>
       <c r="AG183" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -23088,7 +23088,7 @@
       </c>
       <c r="AG184" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -23211,7 +23211,7 @@
       </c>
       <c r="AG185" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -23334,7 +23334,7 @@
       </c>
       <c r="AG186" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -23457,7 +23457,7 @@
       </c>
       <c r="AG187" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -23580,7 +23580,7 @@
       </c>
       <c r="AG188" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -23703,7 +23703,7 @@
       </c>
       <c r="AG189" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -23826,7 +23826,7 @@
       </c>
       <c r="AG190" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -23949,7 +23949,7 @@
       </c>
       <c r="AG191" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -24072,7 +24072,7 @@
       </c>
       <c r="AG192" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -24195,7 +24195,7 @@
       </c>
       <c r="AG193" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -24318,7 +24318,7 @@
       </c>
       <c r="AG194" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -24441,7 +24441,7 @@
       </c>
       <c r="AG195" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -24564,7 +24564,7 @@
       </c>
       <c r="AG196" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -24687,7 +24687,7 @@
       </c>
       <c r="AG197" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -24810,7 +24810,7 @@
       </c>
       <c r="AG198" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -24933,7 +24933,7 @@
       </c>
       <c r="AG199" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -25056,7 +25056,7 @@
       </c>
       <c r="AG200" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -25179,7 +25179,7 @@
       </c>
       <c r="AG201" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -25302,7 +25302,7 @@
       </c>
       <c r="AG202" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -25425,7 +25425,7 @@
       </c>
       <c r="AG203" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -25548,7 +25548,7 @@
       </c>
       <c r="AG204" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -25671,7 +25671,7 @@
       </c>
       <c r="AG205" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -25794,7 +25794,7 @@
       </c>
       <c r="AG206" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -25917,7 +25917,7 @@
       </c>
       <c r="AG207" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -26040,7 +26040,7 @@
       </c>
       <c r="AG208" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -26163,7 +26163,7 @@
       </c>
       <c r="AG209" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -26286,7 +26286,7 @@
       </c>
       <c r="AG210" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -26409,7 +26409,7 @@
       </c>
       <c r="AG211" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -26532,7 +26532,7 @@
       </c>
       <c r="AG212" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -26655,7 +26655,7 @@
       </c>
       <c r="AG213" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -26778,7 +26778,7 @@
       </c>
       <c r="AG214" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -26901,7 +26901,7 @@
       </c>
       <c r="AG215" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -27024,7 +27024,7 @@
       </c>
       <c r="AG216" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -27147,7 +27147,7 @@
       </c>
       <c r="AG217" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -27270,7 +27270,7 @@
       </c>
       <c r="AG218" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -27393,7 +27393,7 @@
       </c>
       <c r="AG219" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -27516,7 +27516,7 @@
       </c>
       <c r="AG220" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -27639,7 +27639,7 @@
       </c>
       <c r="AG221" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -27762,7 +27762,7 @@
       </c>
       <c r="AG222" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -27885,7 +27885,7 @@
       </c>
       <c r="AG223" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -28008,7 +28008,7 @@
       </c>
       <c r="AG224" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -28131,7 +28131,7 @@
       </c>
       <c r="AG225" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -28254,7 +28254,7 @@
       </c>
       <c r="AG226" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -28377,7 +28377,7 @@
       </c>
       <c r="AG227" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -28500,7 +28500,7 @@
       </c>
       <c r="AG228" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -28623,7 +28623,7 @@
       </c>
       <c r="AG229" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -28746,7 +28746,7 @@
       </c>
       <c r="AG230" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -28869,7 +28869,7 @@
       </c>
       <c r="AG231" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -28992,7 +28992,7 @@
       </c>
       <c r="AG232" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -29115,7 +29115,7 @@
       </c>
       <c r="AG233" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -29238,7 +29238,7 @@
       </c>
       <c r="AG234" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -29361,7 +29361,7 @@
       </c>
       <c r="AG235" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -29484,7 +29484,7 @@
       </c>
       <c r="AG236" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -29607,7 +29607,7 @@
       </c>
       <c r="AG237" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -29730,7 +29730,7 @@
       </c>
       <c r="AG238" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -29853,7 +29853,7 @@
       </c>
       <c r="AG239" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -29976,7 +29976,7 @@
       </c>
       <c r="AG240" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -30099,7 +30099,7 @@
       </c>
       <c r="AG241" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -30222,7 +30222,7 @@
       </c>
       <c r="AG242" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -30345,7 +30345,7 @@
       </c>
       <c r="AG243" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -30468,7 +30468,7 @@
       </c>
       <c r="AG244" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -30591,7 +30591,7 @@
       </c>
       <c r="AG245" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -30714,7 +30714,7 @@
       </c>
       <c r="AG246" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -30837,7 +30837,7 @@
       </c>
       <c r="AG247" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -30960,7 +30960,7 @@
       </c>
       <c r="AG248" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -31083,7 +31083,7 @@
       </c>
       <c r="AG249" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -31206,7 +31206,7 @@
       </c>
       <c r="AG250" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -31329,7 +31329,7 @@
       </c>
       <c r="AG251" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -31452,7 +31452,7 @@
       </c>
       <c r="AG252" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -31575,7 +31575,7 @@
       </c>
       <c r="AG253" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -31698,7 +31698,7 @@
       </c>
       <c r="AG254" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -31821,7 +31821,7 @@
       </c>
       <c r="AG255" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -31944,7 +31944,7 @@
       </c>
       <c r="AG256" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -32067,7 +32067,7 @@
       </c>
       <c r="AG257" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -32190,7 +32190,7 @@
       </c>
       <c r="AG258" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -32313,7 +32313,7 @@
       </c>
       <c r="AG259" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -32436,7 +32436,7 @@
       </c>
       <c r="AG260" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -32559,7 +32559,7 @@
       </c>
       <c r="AG261" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -32682,7 +32682,7 @@
       </c>
       <c r="AG262" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -32805,7 +32805,7 @@
       </c>
       <c r="AG263" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -32928,7 +32928,7 @@
       </c>
       <c r="AG264" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -33051,7 +33051,7 @@
       </c>
       <c r="AG265" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -33174,7 +33174,7 @@
       </c>
       <c r="AG266" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -33297,7 +33297,7 @@
       </c>
       <c r="AG267" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -33420,7 +33420,7 @@
       </c>
       <c r="AG268" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>
@@ -33543,7 +33543,7 @@
       </c>
       <c r="AG269" t="inlineStr">
         <is>
-          <t>19/02/2026 16:10:04</t>
+          <t>20/02/2026 07:06:55</t>
         </is>
       </c>
     </row>

</xml_diff>